<commit_message>
Update to growth rates for all countries
</commit_message>
<xml_diff>
--- a/data/country_parameters.xlsx
+++ b/data/country_parameters.xlsx
@@ -8,16 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/viola/Documents/GitHub/global_justice/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DDA481-DAE3-6347-9A2B-37B02C1C7896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22841266-BEA5-9D42-9DBB-65B9963D66AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25600" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
     <sheet name="variables" sheetId="2" r:id="rId2"/>
     <sheet name="notes" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1338,7 +1351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1354,10 +1367,11 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1709,13 +1723,13 @@
       <c r="M1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="11" t="s">
         <v>401</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="11" t="s">
         <v>403</v>
       </c>
       <c r="Q1" s="9" t="s">
@@ -1909,6 +1923,16 @@
       <c r="M2" s="3">
         <v>3</v>
       </c>
+      <c r="N2" s="12">
+        <v>0.7</v>
+      </c>
+      <c r="O2">
+        <v>-1.33</v>
+      </c>
+      <c r="P2" s="13">
+        <f>N2-O2</f>
+        <v>2.0300000000000002</v>
+      </c>
       <c r="Q2" s="3">
         <v>-0.112548169707489</v>
       </c>
@@ -2100,6 +2124,16 @@
       <c r="M3" s="3">
         <v>3</v>
       </c>
+      <c r="N3" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="O3">
+        <v>0.03</v>
+      </c>
+      <c r="P3" s="13">
+        <f t="shared" ref="P3:P16" si="0">N3-O3</f>
+        <v>2.4700000000000002</v>
+      </c>
       <c r="Q3" s="3">
         <v>-0.13730346598477899</v>
       </c>
@@ -2297,7 +2331,8 @@
       <c r="O4">
         <v>-0.65</v>
       </c>
-      <c r="P4" s="11">
+      <c r="P4" s="13">
+        <f t="shared" si="0"/>
         <v>3.94</v>
       </c>
       <c r="Q4" s="3">
@@ -2491,9 +2526,16 @@
       <c r="M5" s="3">
         <v>6</v>
       </c>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
+      <c r="N5" s="3">
+        <v>6.51</v>
+      </c>
+      <c r="O5" s="3">
+        <v>0.83</v>
+      </c>
+      <c r="P5" s="13">
+        <f t="shared" si="0"/>
+        <v>5.68</v>
+      </c>
       <c r="Q5" s="3">
         <v>-9.4905323822841101E-2</v>
       </c>
@@ -2685,9 +2727,16 @@
       <c r="M6" s="3">
         <v>3</v>
       </c>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
+      <c r="N6" s="3">
+        <v>1.76</v>
+      </c>
+      <c r="O6" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="P6" s="13">
+        <f t="shared" si="0"/>
+        <v>1.54</v>
+      </c>
       <c r="Q6" s="3">
         <v>-0.13354093838377301</v>
       </c>
@@ -2879,9 +2928,16 @@
       <c r="M7" s="3">
         <v>2</v>
       </c>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
+      <c r="N7" s="3">
+        <v>1.75</v>
+      </c>
+      <c r="O7" s="3">
+        <v>0.32</v>
+      </c>
+      <c r="P7" s="13">
+        <f t="shared" si="0"/>
+        <v>1.43</v>
+      </c>
       <c r="Q7" s="3">
         <v>-0.12249359204546099</v>
       </c>
@@ -3073,9 +3129,16 @@
       <c r="M8" s="3">
         <v>3</v>
       </c>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
+      <c r="N8" s="3">
+        <v>0.62</v>
+      </c>
+      <c r="O8" s="3">
+        <v>-1</v>
+      </c>
+      <c r="P8" s="13">
+        <f t="shared" si="0"/>
+        <v>1.62</v>
+      </c>
       <c r="Q8" s="3">
         <v>-7.07784864996618E-2</v>
       </c>
@@ -3267,8 +3330,9 @@
       <c r="O9" s="3">
         <v>0.8</v>
       </c>
-      <c r="P9" s="3">
-        <v>2</v>
+      <c r="P9" s="13">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999998</v>
       </c>
       <c r="Q9" s="3"/>
       <c r="R9" t="s">
@@ -3399,9 +3463,16 @@
       <c r="M10" s="3">
         <v>3</v>
       </c>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
+      <c r="N10" s="3">
+        <v>0.61</v>
+      </c>
+      <c r="O10" s="3">
+        <v>-0.7</v>
+      </c>
+      <c r="P10" s="13">
+        <f t="shared" si="0"/>
+        <v>1.31</v>
+      </c>
       <c r="Q10" s="3">
         <v>-0.123622202919661</v>
       </c>
@@ -3593,9 +3664,16 @@
       <c r="M11" s="3">
         <v>2</v>
       </c>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
+      <c r="N11" s="3">
+        <v>2.33</v>
+      </c>
+      <c r="O11" s="3">
+        <v>0.63</v>
+      </c>
+      <c r="P11" s="13">
+        <f t="shared" si="0"/>
+        <v>1.7000000000000002</v>
+      </c>
       <c r="Q11" s="3">
         <v>-0.131534447004375</v>
       </c>
@@ -3787,9 +3865,16 @@
       <c r="M12" s="3">
         <v>3</v>
       </c>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
+      <c r="N12" s="3">
+        <v>1.89</v>
+      </c>
+      <c r="O12" s="3">
+        <v>-1.1299999999999999</v>
+      </c>
+      <c r="P12" s="13">
+        <f t="shared" si="0"/>
+        <v>3.0199999999999996</v>
+      </c>
       <c r="Q12" s="3">
         <v>-0.13219290830986699</v>
       </c>
@@ -3981,9 +4066,16 @@
       <c r="M13" s="3">
         <v>6</v>
       </c>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
+      <c r="N13" s="3">
+        <v>5.23</v>
+      </c>
+      <c r="O13" s="3">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="P13" s="13">
+        <f t="shared" si="0"/>
+        <v>4.6500000000000004</v>
+      </c>
       <c r="Q13" s="3">
         <v>-7.7349779570002095E-2</v>
       </c>
@@ -4175,9 +4267,16 @@
       <c r="M14" s="3">
         <v>3</v>
       </c>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
+      <c r="N14" s="3">
+        <v>1.81</v>
+      </c>
+      <c r="O14" s="3">
+        <v>0.86</v>
+      </c>
+      <c r="P14" s="13">
+        <f t="shared" si="0"/>
+        <v>0.95000000000000007</v>
+      </c>
       <c r="Q14" s="3">
         <v>-6.42063015610502E-2</v>
       </c>
@@ -4369,9 +4468,16 @@
       <c r="M15" s="3">
         <v>4</v>
       </c>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
+      <c r="N15" s="3">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="O15" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="P15" s="13">
+        <f t="shared" si="0"/>
+        <v>3.7199999999999998</v>
+      </c>
       <c r="Q15" s="3">
         <v>-0.153204834852223</v>
       </c>
@@ -4563,9 +4669,16 @@
       <c r="M16" s="3">
         <v>6</v>
       </c>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
+      <c r="N16" s="3">
+        <v>4.18</v>
+      </c>
+      <c r="O16" s="3">
+        <v>2.62</v>
+      </c>
+      <c r="P16" s="13">
+        <f t="shared" si="0"/>
+        <v>1.5599999999999996</v>
+      </c>
       <c r="Q16" s="3">
         <v>-6.0798141137966402E-2</v>
       </c>

</xml_diff>

<commit_message>
Update with beef and flights numbers
</commit_message>
<xml_diff>
--- a/data/country_parameters.xlsx
+++ b/data/country_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/viola/Documents/GitHub/global_justice/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22841266-BEA5-9D42-9DBB-65B9963D66AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7432F7B-5767-5C48-8483-30C2347C1832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25600" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="411">
   <si>
     <t>note</t>
   </si>
@@ -1247,6 +1247,27 @@
   </si>
   <si>
     <t>GDP/worker growth 2031 g(GDP)-g(labour force)</t>
+  </si>
+  <si>
+    <t>beef consumption kg/cp/yr 2026_OECD-FAO Agricultural Outlook 2024-2033</t>
+  </si>
+  <si>
+    <t>beef target 2100 (Chancel)</t>
+  </si>
+  <si>
+    <t>beef cons variation over 2026-2100</t>
+  </si>
+  <si>
+    <t>aviation CO2 (kg/cp/yr) 2024_OWID</t>
+  </si>
+  <si>
+    <t>aviation target: 2024  World average (kg/cp/yr)_OWID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aviation cons variation </t>
+  </si>
+  <si>
+    <t>EU average</t>
   </si>
 </sst>
 </file>
@@ -1258,7 +1279,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1287,8 +1308,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1329,8 +1358,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1347,11 +1382,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1370,8 +1414,18 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1668,7 +1722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BN31"/>
+  <dimension ref="A1:BU31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="6.6640625" customWidth="1"/>
@@ -1683,7 +1737,7 @@
     <col min="21" max="66" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="59" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:73" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>12</v>
       </c>
@@ -1882,8 +1936,27 @@
       <c r="BN1" s="9" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="2" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO1" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="BP1" s="13"/>
+      <c r="BQ1" s="14" t="s">
+        <v>405</v>
+      </c>
+      <c r="BR1" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="BS1" s="15" t="s">
+        <v>407</v>
+      </c>
+      <c r="BT1" s="15" t="s">
+        <v>408</v>
+      </c>
+      <c r="BU1" s="15" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="2" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -1923,13 +1996,13 @@
       <c r="M2" s="3">
         <v>3</v>
       </c>
-      <c r="N2" s="12">
+      <c r="N2" s="3">
         <v>0.7</v>
       </c>
       <c r="O2">
         <v>-1.33</v>
       </c>
-      <c r="P2" s="13">
+      <c r="P2" s="12">
         <f>N2-O2</f>
         <v>2.0300000000000002</v>
       </c>
@@ -2083,8 +2156,31 @@
       <c r="BN2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO2" s="12">
+        <v>9.2200000000000006</v>
+      </c>
+      <c r="BP2" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="BQ2">
+        <v>5.9</v>
+      </c>
+      <c r="BR2" s="12">
+        <f>(BQ2/BO2-1)</f>
+        <v>-0.36008676789587857</v>
+      </c>
+      <c r="BS2" s="12">
+        <v>240.62</v>
+      </c>
+      <c r="BT2" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU2" s="12">
+        <f>(BT2/BS2-1)</f>
+        <v>-0.57725874823372947</v>
+      </c>
+    </row>
+    <row r="3" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -2124,13 +2220,13 @@
       <c r="M3" s="3">
         <v>3</v>
       </c>
-      <c r="N3" s="12">
+      <c r="N3" s="3">
         <v>2.5</v>
       </c>
       <c r="O3">
         <v>0.03</v>
       </c>
-      <c r="P3" s="13">
+      <c r="P3" s="12">
         <f t="shared" ref="P3:P16" si="0">N3-O3</f>
         <v>2.4700000000000002</v>
       </c>
@@ -2284,8 +2380,29 @@
       <c r="BN3">
         <v>1.004</v>
       </c>
-    </row>
-    <row r="4" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO3" s="16">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="BP3" s="12"/>
+      <c r="BQ3">
+        <v>5.9</v>
+      </c>
+      <c r="BR3" s="12">
+        <f t="shared" ref="BR3:BR16" si="1">(BQ3/BO3-1)</f>
+        <v>-0.68783068783068779</v>
+      </c>
+      <c r="BS3" s="12">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="BT3" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU3" s="17">
+        <f t="shared" ref="BU3:BU16" si="2">(BT3/BS3-1)</f>
+        <v>0.37645466847090647</v>
+      </c>
+    </row>
+    <row r="4" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>82</v>
       </c>
@@ -2331,7 +2448,7 @@
       <c r="O4">
         <v>-0.65</v>
       </c>
-      <c r="P4" s="13">
+      <c r="P4" s="12">
         <f t="shared" si="0"/>
         <v>3.94</v>
       </c>
@@ -2485,8 +2602,29 @@
       <c r="BN4">
         <v>0.96099999999999997</v>
       </c>
-    </row>
-    <row r="5" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO4" s="12">
+        <v>4.99</v>
+      </c>
+      <c r="BP4" s="12"/>
+      <c r="BQ4">
+        <v>5.9</v>
+      </c>
+      <c r="BR4" s="17">
+        <f t="shared" si="1"/>
+        <v>0.18236472945891791</v>
+      </c>
+      <c r="BS4" s="12">
+        <v>74.58</v>
+      </c>
+      <c r="BT4" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU4" s="17">
+        <f t="shared" si="2"/>
+        <v>0.36390453204612494</v>
+      </c>
+    </row>
+    <row r="5" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -2532,7 +2670,7 @@
       <c r="O5" s="3">
         <v>0.83</v>
       </c>
-      <c r="P5" s="13">
+      <c r="P5" s="12">
         <f t="shared" si="0"/>
         <v>5.68</v>
       </c>
@@ -2686,8 +2824,29 @@
       <c r="BN5">
         <v>1.2370000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO5" s="12">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="BP5" s="12"/>
+      <c r="BQ5">
+        <v>5.9</v>
+      </c>
+      <c r="BR5" s="17">
+        <f t="shared" si="1"/>
+        <v>4.2678571428571423</v>
+      </c>
+      <c r="BS5" s="12">
+        <v>17.079999999999998</v>
+      </c>
+      <c r="BT5" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU5" s="17">
+        <f t="shared" si="2"/>
+        <v>4.9555035128805622</v>
+      </c>
+    </row>
+    <row r="6" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -2733,7 +2892,7 @@
       <c r="O6" s="3">
         <v>0.22</v>
       </c>
-      <c r="P6" s="13">
+      <c r="P6" s="12">
         <f t="shared" si="0"/>
         <v>1.54</v>
       </c>
@@ -2887,8 +3046,29 @@
       <c r="BN6">
         <v>1.0640000000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO6" s="12">
+        <v>23.27</v>
+      </c>
+      <c r="BP6" s="12"/>
+      <c r="BQ6">
+        <v>5.9</v>
+      </c>
+      <c r="BR6" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.74645466265577998</v>
+      </c>
+      <c r="BS6" s="12">
+        <v>579.51</v>
+      </c>
+      <c r="BT6" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU6" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.82447239909578784</v>
+      </c>
+    </row>
+    <row r="7" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>98</v>
       </c>
@@ -2934,7 +3114,7 @@
       <c r="O7" s="3">
         <v>0.32</v>
       </c>
-      <c r="P7" s="13">
+      <c r="P7" s="12">
         <f t="shared" si="0"/>
         <v>1.43</v>
       </c>
@@ -3088,8 +3268,29 @@
       <c r="BN7">
         <v>1.0669999999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO7" s="12">
+        <v>17.27</v>
+      </c>
+      <c r="BP7" s="12"/>
+      <c r="BQ7">
+        <v>5.9</v>
+      </c>
+      <c r="BR7" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.65836711059640995</v>
+      </c>
+      <c r="BS7" s="12">
+        <v>474.21</v>
+      </c>
+      <c r="BT7" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU7" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.78549587735391491</v>
+      </c>
+    </row>
+    <row r="8" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>103</v>
       </c>
@@ -3135,7 +3336,7 @@
       <c r="O8" s="3">
         <v>-1</v>
       </c>
-      <c r="P8" s="13">
+      <c r="P8" s="12">
         <f t="shared" si="0"/>
         <v>1.62</v>
       </c>
@@ -3289,8 +3490,31 @@
       <c r="BN8">
         <v>0.99399999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO8" s="12">
+        <v>9.2200000000000006</v>
+      </c>
+      <c r="BP8" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="BQ8">
+        <v>5.9</v>
+      </c>
+      <c r="BR8" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.36008676789587857</v>
+      </c>
+      <c r="BS8" s="12">
+        <v>256.83999999999997</v>
+      </c>
+      <c r="BT8" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU8" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.60395577012926327</v>
+      </c>
+    </row>
+    <row r="9" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>107</v>
       </c>
@@ -3330,7 +3554,7 @@
       <c r="O9" s="3">
         <v>0.8</v>
       </c>
-      <c r="P9" s="13">
+      <c r="P9" s="12">
         <f t="shared" si="0"/>
         <v>1.9999999999999998</v>
       </c>
@@ -3422,8 +3646,29 @@
       <c r="BN9">
         <v>1.0720000000000001</v>
       </c>
-    </row>
-    <row r="10" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO9" s="12">
+        <v>3.88</v>
+      </c>
+      <c r="BP9" s="12"/>
+      <c r="BQ9">
+        <v>5.9</v>
+      </c>
+      <c r="BR9" s="17">
+        <f t="shared" si="1"/>
+        <v>0.52061855670103108</v>
+      </c>
+      <c r="BS9" s="12">
+        <v>77.349999999999994</v>
+      </c>
+      <c r="BT9" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU9" s="17">
+        <f t="shared" si="2"/>
+        <v>0.31506140917905623</v>
+      </c>
+    </row>
+    <row r="10" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>113</v>
       </c>
@@ -3469,7 +3714,7 @@
       <c r="O10" s="3">
         <v>-0.7</v>
       </c>
-      <c r="P10" s="13">
+      <c r="P10" s="12">
         <f t="shared" si="0"/>
         <v>1.31</v>
       </c>
@@ -3623,8 +3868,29 @@
       <c r="BN10">
         <v>1.0680000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO10" s="12">
+        <v>7.05</v>
+      </c>
+      <c r="BP10" s="12"/>
+      <c r="BQ10">
+        <v>5.9</v>
+      </c>
+      <c r="BR10" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.16312056737588643</v>
+      </c>
+      <c r="BS10" s="12">
+        <v>221.34</v>
+      </c>
+      <c r="BT10" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU10" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.54043552905032977</v>
+      </c>
+    </row>
+    <row r="11" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>118</v>
       </c>
@@ -3670,7 +3936,7 @@
       <c r="O11" s="3">
         <v>0.63</v>
       </c>
-      <c r="P11" s="13">
+      <c r="P11" s="12">
         <f t="shared" si="0"/>
         <v>1.7000000000000002</v>
       </c>
@@ -3824,8 +4090,29 @@
       <c r="BN11">
         <v>0.98799999999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO11" s="12">
+        <v>23.01</v>
+      </c>
+      <c r="BP11" s="12"/>
+      <c r="BQ11">
+        <v>5.9</v>
+      </c>
+      <c r="BR11" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.74358974358974361</v>
+      </c>
+      <c r="BS11" s="12">
+        <v>759.01</v>
+      </c>
+      <c r="BT11" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU11" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.86598332037786063</v>
+      </c>
+    </row>
+    <row r="12" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -3871,7 +4158,7 @@
       <c r="O12" s="3">
         <v>-1.1299999999999999</v>
       </c>
-      <c r="P12" s="13">
+      <c r="P12" s="12">
         <f t="shared" si="0"/>
         <v>3.0199999999999996</v>
       </c>
@@ -4025,8 +4312,29 @@
       <c r="BN12">
         <v>1.081</v>
       </c>
-    </row>
-    <row r="13" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO12" s="12">
+        <v>12.28</v>
+      </c>
+      <c r="BP12" s="12"/>
+      <c r="BQ12">
+        <v>5.9</v>
+      </c>
+      <c r="BR12" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.51954397394136809</v>
+      </c>
+      <c r="BS12" s="12">
+        <v>285.36</v>
+      </c>
+      <c r="BT12" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU12" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.643537987104009</v>
+      </c>
+    </row>
+    <row r="13" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>129</v>
       </c>
@@ -4072,7 +4380,7 @@
       <c r="O13" s="3">
         <v>0.57999999999999996</v>
       </c>
-      <c r="P13" s="13">
+      <c r="P13" s="12">
         <f t="shared" si="0"/>
         <v>4.6500000000000004</v>
       </c>
@@ -4226,8 +4534,29 @@
       <c r="BN13">
         <v>1.135</v>
       </c>
-    </row>
-    <row r="14" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO13" s="12">
+        <v>1.67</v>
+      </c>
+      <c r="BP13" s="12"/>
+      <c r="BQ13">
+        <v>5.9</v>
+      </c>
+      <c r="BR13" s="17">
+        <f t="shared" si="1"/>
+        <v>2.5329341317365275</v>
+      </c>
+      <c r="BS13" s="12">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="BT13" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU13" s="17">
+        <f t="shared" si="2"/>
+        <v>1.7270777479892763</v>
+      </c>
+    </row>
+    <row r="14" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>134</v>
       </c>
@@ -4273,7 +4602,7 @@
       <c r="O14" s="3">
         <v>0.86</v>
       </c>
-      <c r="P14" s="13">
+      <c r="P14" s="12">
         <f t="shared" si="0"/>
         <v>0.95000000000000007</v>
       </c>
@@ -4427,8 +4756,29 @@
       <c r="BN14">
         <v>0.96799999999999997</v>
       </c>
-    </row>
-    <row r="15" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO14" s="12">
+        <v>10.16</v>
+      </c>
+      <c r="BP14" s="12"/>
+      <c r="BQ14">
+        <v>5.9</v>
+      </c>
+      <c r="BR14" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.41929133858267709</v>
+      </c>
+      <c r="BS14" s="12">
+        <v>72.17</v>
+      </c>
+      <c r="BT14" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU14" s="17">
+        <f t="shared" si="2"/>
+        <v>0.40944990993487584</v>
+      </c>
+    </row>
+    <row r="15" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>140</v>
       </c>
@@ -4474,7 +4824,7 @@
       <c r="O15" s="3">
         <v>0.3</v>
       </c>
-      <c r="P15" s="13">
+      <c r="P15" s="12">
         <f t="shared" si="0"/>
         <v>3.7199999999999998</v>
       </c>
@@ -4628,8 +4978,29 @@
       <c r="BN15">
         <v>2.4580000000000002</v>
       </c>
-    </row>
-    <row r="16" spans="1:66" x14ac:dyDescent="0.2">
+      <c r="BO15" s="12">
+        <v>11.83</v>
+      </c>
+      <c r="BP15" s="12"/>
+      <c r="BQ15">
+        <v>5.9</v>
+      </c>
+      <c r="BR15" s="12">
+        <f t="shared" si="1"/>
+        <v>-0.50126796280642427</v>
+      </c>
+      <c r="BS15" s="12">
+        <v>198.4</v>
+      </c>
+      <c r="BT15" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU15" s="12">
+        <f t="shared" si="2"/>
+        <v>-0.4872983870967742</v>
+      </c>
+    </row>
+    <row r="16" spans="1:73" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>145</v>
       </c>
@@ -4675,7 +5046,7 @@
       <c r="O16" s="3">
         <v>2.62</v>
       </c>
-      <c r="P16" s="13">
+      <c r="P16" s="12">
         <f t="shared" si="0"/>
         <v>1.5599999999999996</v>
       </c>
@@ -4828,6 +5199,27 @@
       </c>
       <c r="BN16">
         <v>1.137</v>
+      </c>
+      <c r="BO16" s="12">
+        <v>0.87080000000000002</v>
+      </c>
+      <c r="BP16" s="12"/>
+      <c r="BQ16">
+        <v>5.9</v>
+      </c>
+      <c r="BR16" s="17">
+        <f t="shared" si="1"/>
+        <v>5.7753789618741393</v>
+      </c>
+      <c r="BS16" s="12">
+        <v>4.62</v>
+      </c>
+      <c r="BT16" s="12">
+        <v>101.72</v>
+      </c>
+      <c r="BU16" s="17">
+        <f t="shared" si="2"/>
+        <v>21.017316017316016</v>
       </c>
     </row>
     <row r="17" spans="1:66" x14ac:dyDescent="0.2">

</xml_diff>